<commit_message>
Improve evaluation Excel with screenshot-ready Dashboard Index sheet
Co-authored-by: zainabbastahirag <zainabbastahirag@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/candidate_evaluation.xlsx
+++ b/candidate_evaluation.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Phase 1 Scores" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Phase 2 Scores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dashboard Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Session 1 — Phase 1 Scores" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Session 2 — Phase 2 Scores" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Phase 1 — Detailed Notes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Phase 2 — Detailed Notes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Summary" sheetId="6" state="visible" r:id="rId6"/>
@@ -33,25 +33,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -63,7 +51,18 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00000000"/>
-      <sz val="14"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -72,7 +71,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -86,7 +85,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,7 +105,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E2F3"/>
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2DFEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,54 +145,104 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -535,112 +604,525 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Candidate Evaluation — Phase 1 &amp; Phase 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr"/>
+          <t>CANDIDATE EVALUATION — DASHBOARD INDEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1 = Weak  |  2 = Below avg  |  3 = Average  |  4 = Good  |  5 = Excellent</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Session 1 — Phase 1</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Presentation + Technical Observation</t>
+          <t>SESSION 1 — PHASE 1  |  Presentation + Technical Observation</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Candidates</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Mohammad Kashif Mohiuddin, Shahid, Hadeef</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Technical Observation</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Strengths</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="A6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Kashif Mohiuddin</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="7">
+        <f>SUM(C6:D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="7">
+        <f>IF(COUNT(C6:D6)&gt;0,AVERAGE(C6:D6),"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Session 2 — Phase 2</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Clarity &amp; discussion criteria (simplified labels)</t>
-        </is>
-      </c>
+      <c r="A7" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Shahid</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="10">
+        <f>SUM(C7:D7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="10">
+        <f>IF(COUNT(C7:D7)&gt;0,AVERAGE(C7:D7),"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Candidates</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Baizid Yaldram, MUHAMMAD HADIF AMAR BIN RAZALI, CITA WAFA ATIAH, MUHAMMAD MAIRAJ, Mohammad Shahid Akhtar, Aurneela Ghosh Riddhi</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="A8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Hadeef</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="7">
+        <f>SUM(C8:D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="7">
+        <f>IF(COUNT(C8:D8)&gt;0,AVERAGE(C8:D8),"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Rating scale</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>1 = Weak | 2 = Below avg | 3 = Average | 4 = Good | 5 = Excellent</t>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>SESSION 2 — PHASE 2  |  Clarity &amp; Discussion (simple labels)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Clear Thinking</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Deep vs Wide</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Build on Ideas</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Business Link</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Positive Manner</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Fresh Ideas</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Speaking Style</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>Strengths</t>
+        </is>
+      </c>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Sheets</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Phase 1 Scores | Phase 2 Scores | Phase 1 Notes | Phase 2 Notes | Summary</t>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Baizid Yaldram</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="7">
+        <f>SUM(C12:I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="7">
+        <f>IF(COUNT(C12:I12)&gt;0,AVERAGE(C12:I12),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="14" t="n"/>
+      <c r="M12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>MUHAMMAD HADIF AMAR BIN RAZALI</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="10">
+        <f>SUM(C13:I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="10">
+        <f>IF(COUNT(C13:I13)&gt;0,AVERAGE(C13:I13),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="16" t="n"/>
+      <c r="M13" s="16" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>CITA WAFA ATIAH</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="7">
+        <f>SUM(C14:I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="7">
+        <f>IF(COUNT(C14:I14)&gt;0,AVERAGE(C14:I14),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="14" t="n"/>
+      <c r="M14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>MUHAMMAD MAIRAJ</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="10">
+        <f>SUM(C15:I15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="10">
+        <f>IF(COUNT(C15:I15)&gt;0,AVERAGE(C15:I15),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="16" t="n"/>
+      <c r="M15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Mohammad Shahid Akhtar</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="7">
+        <f>SUM(C16:I16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="7">
+        <f>IF(COUNT(C16:I16)&gt;0,AVERAGE(C16:I16),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="14" t="n"/>
+      <c r="M16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Aurneela Ghosh Riddhi</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="10">
+        <f>SUM(C17:I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="10">
+        <f>IF(COUNT(C17:I17)&gt;0,AVERAGE(C17:I17),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="16" t="n"/>
+      <c r="M17" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>PHASE 2 CRITERIA GUIDE (simple words)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Clear Thinking</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Deep vs Wide</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Build on Ideas</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Business Link</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Positive Manner</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Fresh Ideas</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Speaking Style</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="12">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B23:H23"/>
   </mergeCells>
+  <conditionalFormatting sqref="C6:D8">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThanOrEqual" dxfId="2">
+      <formula>2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12:I17">
+    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="0">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="lessThanOrEqual" dxfId="2">
+      <formula>2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="C6 C7 C8 D6 D7 D8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid score" error="Enter a score from 1 to 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12 C13 C14 C15 C16 C17 D12 D13 D14 D15 D16 D17 E12 E13 E14 E15 E16 E17 F12 F13 F14 F15 F16 F17 G12 G13 G14 G15 G16 G17 H12 H13 H14 H15 H16 H17 I12 I13 I14 I15 I16 I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid score" error="Enter a score from 1 to 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -651,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -663,63 +1145,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>SESSION 1 — PHASE 1 SCORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Candidate</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Presentation</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Technical Observation</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Overall Notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Mohammad Kashif Mohiuddin</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="7">
-        <f>SUM(B2:C2)</f>
-        <v/>
-      </c>
-      <c r="E2" s="7">
-        <f>IF(COUNT(B2:C2)&gt;0,AVERAGE(B2:C2),"")</f>
-        <v/>
-      </c>
-      <c r="F2" s="5" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Shahid</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
       <c r="D3" s="10">
         <f>SUM(B3:C3)</f>
         <v/>
@@ -728,16 +1199,16 @@
         <f>IF(COUNT(B3:C3)&gt;0,AVERAGE(B3:C3),"")</f>
         <v/>
       </c>
-      <c r="F3" s="8" t="n"/>
+      <c r="F3" s="9" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Hadeef</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Shahid</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
       <c r="D4" s="7">
         <f>SUM(B4:C4)</f>
         <v/>
@@ -746,36 +1217,71 @@
         <f>IF(COUNT(B4:C4)&gt;0,AVERAGE(B4:C4),"")</f>
         <v/>
       </c>
-      <c r="F4" s="5" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="F4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Hadeef</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="10">
+        <f>SUM(B5:C5)</f>
+        <v/>
+      </c>
+      <c r="E5" s="10">
+        <f>IF(COUNT(B5:C5)&gt;0,AVERAGE(B5:C5),"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Criteria guide</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Presentation: How well they present — structure, confidence, slides, delivery</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Technical Observation: How well they spot and explain technical points</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>1 = Weak | 2 = Below avg | 3 = Average | 4 = Good | 5 = Excellent</t>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Presentation: Structure, confidence, slides, delivery</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Technical Observation: Spots and explains technical points well</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>1 = Weak  |  2 = Below avg  |  3 = Average  |  4 = Good  |  5 = Excellent</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A7:F7"/>
+  <mergeCells count="2">
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:C5">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThanOrEqual" dxfId="2">
+      <formula>2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B3 B4 B5 C3 C4 C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid score" error="Enter a score from 1 to 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -786,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -803,98 +1309,82 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>SESSION 2 — PHASE 2 SCORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Candidate</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J2" s="23" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>Overall Notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Baizid Yaldram</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7">
-        <f>SUM(B2:H2)</f>
-        <v/>
-      </c>
-      <c r="J2" s="7">
-        <f>IF(COUNT(B2:H2)&gt;0,AVERAGE(B2:H2),"")</f>
-        <v/>
-      </c>
-      <c r="K2" s="5" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>MUHAMMAD HADIF AMAR BIN RAZALI</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
       <c r="I3" s="10">
         <f>SUM(B3:H3)</f>
         <v/>
@@ -903,21 +1393,21 @@
         <f>IF(COUNT(B3:H3)&gt;0,AVERAGE(B3:H3),"")</f>
         <v/>
       </c>
-      <c r="K3" s="8" t="n"/>
+      <c r="K3" s="9" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>CITA WAFA ATIAH</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>MUHAMMAD HADIF AMAR BIN RAZALI</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
       <c r="I4" s="7">
         <f>SUM(B4:H4)</f>
         <v/>
@@ -926,21 +1416,21 @@
         <f>IF(COUNT(B4:H4)&gt;0,AVERAGE(B4:H4),"")</f>
         <v/>
       </c>
-      <c r="K4" s="5" t="n"/>
+      <c r="K4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>MUHAMMAD MAIRAJ</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>CITA WAFA ATIAH</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
       <c r="I5" s="10">
         <f>SUM(B5:H5)</f>
         <v/>
@@ -949,21 +1439,21 @@
         <f>IF(COUNT(B5:H5)&gt;0,AVERAGE(B5:H5),"")</f>
         <v/>
       </c>
-      <c r="K5" s="8" t="n"/>
+      <c r="K5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Mohammad Shahid Akhtar</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>MUHAMMAD MAIRAJ</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
       <c r="I6" s="7">
         <f>SUM(B6:H6)</f>
         <v/>
@@ -972,21 +1462,21 @@
         <f>IF(COUNT(B6:H6)&gt;0,AVERAGE(B6:H6),"")</f>
         <v/>
       </c>
-      <c r="K6" s="5" t="n"/>
+      <c r="K6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Aurneela Ghosh Riddhi</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Mohammad Shahid Akhtar</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
       <c r="I7" s="10">
         <f>SUM(B7:H7)</f>
         <v/>
@@ -995,61 +1485,101 @@
         <f>IF(COUNT(B7:H7)&gt;0,AVERAGE(B7:H7),"")</f>
         <v/>
       </c>
-      <c r="K7" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="K7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Aurneela Ghosh Riddhi</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="7">
+        <f>SUM(B8:H8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="7">
+        <f>IF(COUNT(B8:H8)&gt;0,AVERAGE(B8:H8),"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Criteria guide</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Clear Thinking: How easy their ideas are to follow (clarity of thought)</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Deep vs Wide: Goes deep on topics vs covers many areas (depth vs breadth)</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Build on Ideas: Lists points and builds on them step by step (listing &amp; building)</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Business Link: Connects ideas to real business value (business linkage)</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Positive Manner: Respectful, calm, professional conduct (conduct with benefit)</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>Fresh Ideas: Shows own thinking, not just textbook answers (original thinking)</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>Speaking Style: Tone, pace, and how clearly they communicate (communication style)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>1 = Weak | 2 = Below avg | 3 = Average | 4 = Good | 5 = Excellent</t>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Clear Thinking: Clarity of thought — easy to follow</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Deep vs Wide: Depth vs breadth of answers</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Build on Ideas: Listing and building on points</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Business Link: Links ideas to business value</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>Positive Manner: Conduct with benefit — respectful &amp; calm</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Fresh Ideas: Original thinking</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>Speaking Style: Communication style</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>1 = Weak  |  2 = Below avg  |  3 = Average  |  4 = Good  |  5 = Excellent</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A10:K10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:H8">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThanOrEqual" dxfId="2">
+      <formula>2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B3 B4 B5 B6 B7 B8 C3 C4 C5 C6 C7 C8 D3 D4 D5 D6 D7 D8 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 G3 G4 G5 G6 G7 G8 H3 H4 H5 H6 H7 H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid score" error="Enter a score from 1 to 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1070,102 +1600,102 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Phase 1 — Detailed Notes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Mohammad Kashif Mohiuddin</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>(How well they present — structure, confidence, slides, delivery)</t>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Structure, confidence, slides, delivery</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Technical Observation</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>(How well they spot and explain technical points)</t>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Spots and explains technical points well</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Shahid</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>(How well they present — structure, confidence, slides, delivery)</t>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Structure, confidence, slides, delivery</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Technical Observation</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>(How well they spot and explain technical points)</t>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Spots and explains technical points well</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Hadeef</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>(How well they present — structure, confidence, slides, delivery)</t>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Structure, confidence, slides, delivery</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Technical Observation</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>(How well they spot and explain technical points)</t>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Spots and explains technical points well</t>
         </is>
       </c>
     </row>
@@ -1202,555 +1732,555 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Phase 2 — Detailed Notes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Baizid Yaldram</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>(How easy their ideas are to follow (clarity of thought))</t>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>(Goes deep on topics vs covers many areas (depth vs breadth))</t>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>(Lists points and builds on them step by step (listing &amp; building))</t>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>(Connects ideas to real business value (business linkage))</t>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>(Respectful, calm, professional conduct (conduct with benefit))</t>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>(Shows own thinking, not just textbook answers (original thinking))</t>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>(Tone, pace, and how clearly they communicate (communication style))</t>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>MUHAMMAD HADIF AMAR BIN RAZALI</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>(How easy their ideas are to follow (clarity of thought))</t>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>(Goes deep on topics vs covers many areas (depth vs breadth))</t>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>(Lists points and builds on them step by step (listing &amp; building))</t>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>(Connects ideas to real business value (business linkage))</t>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>(Respectful, calm, professional conduct (conduct with benefit))</t>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>(Shows own thinking, not just textbook answers (original thinking))</t>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>(Tone, pace, and how clearly they communicate (communication style))</t>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>CITA WAFA ATIAH</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>(How easy their ideas are to follow (clarity of thought))</t>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>(Goes deep on topics vs covers many areas (depth vs breadth))</t>
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>(Lists points and builds on them step by step (listing &amp; building))</t>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>(Connects ideas to real business value (business linkage))</t>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>(Respectful, calm, professional conduct (conduct with benefit))</t>
+      <c r="B44" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>(Shows own thinking, not just textbook answers (original thinking))</t>
+      <c r="B46" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="18" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>(Tone, pace, and how clearly they communicate (communication style))</t>
+      <c r="B48" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="A51" s="21" t="inlineStr">
         <is>
           <t>MUHAMMAD MAIRAJ</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="A52" s="18" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>(How easy their ideas are to follow (clarity of thought))</t>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="18" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>(Goes deep on topics vs covers many areas (depth vs breadth))</t>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="18" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>(Lists points and builds on them step by step (listing &amp; building))</t>
+      <c r="B56" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="18" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>(Connects ideas to real business value (business linkage))</t>
+      <c r="B58" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="18" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>(Respectful, calm, professional conduct (conduct with benefit))</t>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="18" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>(Shows own thinking, not just textbook answers (original thinking))</t>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+      <c r="A64" s="18" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>(Tone, pace, and how clearly they communicate (communication style))</t>
+      <c r="B64" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="A67" s="21" t="inlineStr">
         <is>
           <t>Mohammad Shahid Akhtar</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="18" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>(How easy their ideas are to follow (clarity of thought))</t>
+      <c r="B68" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+      <c r="A70" s="18" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>(Goes deep on topics vs covers many areas (depth vs breadth))</t>
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+      <c r="A72" s="18" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>(Lists points and builds on them step by step (listing &amp; building))</t>
+      <c r="B72" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr">
+      <c r="A74" s="18" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>(Connects ideas to real business value (business linkage))</t>
+      <c r="B74" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="A76" s="18" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>(Respectful, calm, professional conduct (conduct with benefit))</t>
+      <c r="B76" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="3" t="inlineStr">
+      <c r="A78" s="18" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>(Shows own thinking, not just textbook answers (original thinking))</t>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3" t="inlineStr">
+      <c r="A80" s="18" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>(Tone, pace, and how clearly they communicate (communication style))</t>
+      <c r="B80" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="11" t="inlineStr">
+      <c r="A83" s="21" t="inlineStr">
         <is>
           <t>Aurneela Ghosh Riddhi</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+      <c r="A84" s="18" t="inlineStr">
         <is>
           <t>Clear Thinking</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>(How easy their ideas are to follow (clarity of thought))</t>
+      <c r="B84" s="19" t="inlineStr">
+        <is>
+          <t>Clarity of thought — easy to follow</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="18" t="inlineStr">
         <is>
           <t>Deep vs Wide</t>
         </is>
       </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>(Goes deep on topics vs covers many areas (depth vs breadth))</t>
+      <c r="B86" s="19" t="inlineStr">
+        <is>
+          <t>Depth vs breadth of answers</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="3" t="inlineStr">
+      <c r="A88" s="18" t="inlineStr">
         <is>
           <t>Build on Ideas</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>(Lists points and builds on them step by step (listing &amp; building))</t>
+      <c r="B88" s="19" t="inlineStr">
+        <is>
+          <t>Listing and building on points</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
+      <c r="A90" s="18" t="inlineStr">
         <is>
           <t>Business Link</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>(Connects ideas to real business value (business linkage))</t>
+      <c r="B90" s="19" t="inlineStr">
+        <is>
+          <t>Links ideas to business value</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
+      <c r="A92" s="18" t="inlineStr">
         <is>
           <t>Positive Manner</t>
         </is>
       </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>(Respectful, calm, professional conduct (conduct with benefit))</t>
+      <c r="B92" s="19" t="inlineStr">
+        <is>
+          <t>Conduct with benefit — respectful &amp; calm</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="3" t="inlineStr">
+      <c r="A94" s="18" t="inlineStr">
         <is>
           <t>Fresh Ideas</t>
         </is>
       </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>(Shows own thinking, not just textbook answers (original thinking))</t>
+      <c r="B94" s="19" t="inlineStr">
+        <is>
+          <t>Original thinking</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+      <c r="A96" s="18" t="inlineStr">
         <is>
           <t>Speaking Style</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>(Tone, pace, and how clearly they communicate (communication style))</t>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>Communication style</t>
         </is>
       </c>
     </row>
@@ -1829,206 +2359,211 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>All Candidates — Quick Comparison</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>ALL CANDIDATES — QUICK COMPARISON</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Candidate</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>Avg Score</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>Strengths</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>Areas to improve</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
+      <c r="F2" s="17" t="inlineStr">
         <is>
           <t>Recommend?</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
         <is>
           <t>Final notes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Mohammad Kashif Mohiuddin</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr"/>
-      <c r="D3" s="8" t="inlineStr"/>
-      <c r="E3" s="8" t="inlineStr"/>
-      <c r="F3" s="8" t="inlineStr"/>
-      <c r="G3" s="8" t="inlineStr"/>
+      <c r="C3" s="6" t="inlineStr"/>
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Shahid</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="C4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Hadeef</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr"/>
-      <c r="D5" s="8" t="inlineStr"/>
-      <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr"/>
-      <c r="G5" s="8" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Baizid Yaldram</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>MUHAMMAD HADIF AMAR BIN RAZALI</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr"/>
-      <c r="D7" s="8" t="inlineStr"/>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>CITA WAFA ATIAH</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>MUHAMMAD MAIRAJ</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr"/>
-      <c r="D9" s="8" t="inlineStr"/>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Mohammad Shahid Akhtar</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="5" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Aurneela Ghosh Riddhi</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr"/>
-      <c r="D11" s="8" t="inlineStr"/>
-      <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F3 F4 F5 F6 F7 F8 F9 F10 F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,Maybe,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>